<commit_message>
Web sürümü: Pyodide ile tarayıcıda çalışan statik site (Cloudflare Pages) + tablo tabanlı tesir kesiti
- web/: arayüz (yükleme, numune formu, ayarlar, sonuç sekmeleri, grafik, indirme), worker, yayınlama kılavuzu
- tools/build_web.py ve tools/vendor_pyodide.py: site + zip üretimi (CDN'li küçük, kendi içinde tam sürüm)
- gamma_shielding: EPDL97 tablo backend'i (fisx gerekmez), bileşik/mol% bileşim ayrıştırıcı, web_api, ilerleme geri çağrısı,
  SPC bayt ayrıştırıcı; kullanıcıya dönük mesajlar Türkçe karakterli
- tests: web_api, composition, tablo-fisx uyumu, SPC yazıcı; tests/e2e_web.py (Chromium'da uçtan uca doğrulama)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RdE8Sr4qTJowLpjpf43VQj
</commit_message>
<xml_diff>
--- a/examples/sentetik_ornek/sonuclar.xlsx
+++ b/examples/sentetik_ornek/sonuclar.xlsx
@@ -456,7 +456,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="39" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,7 +663,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spektrumlarda tespit edilemeyen cizgiler (analiz disi birakildi): Am-241 59.5 (en yuksek 0.8 sigma); Co-57 122 (en yuksek 2.5 sigma)</t>
+          <t>Spektrumlarda tespit edilemeyen çizgiler (analiz dışı bırakıldı): Am-241 59.5 (en yüksek 0.8σ); Co-57 122 (en yüksek 2.5σ)</t>
         </is>
       </c>
     </row>
@@ -1607,13 +1607,13 @@
     <col width="20" customWidth="1" min="48" max="48"/>
     <col width="20" customWidth="1" min="49" max="49"/>
     <col width="21" customWidth="1" min="50" max="50"/>
-    <col width="22" customWidth="1" min="51" max="51"/>
+    <col width="21" customWidth="1" min="51" max="51"/>
     <col width="21" customWidth="1" min="52" max="52"/>
     <col width="20" customWidth="1" min="53" max="53"/>
     <col width="24" customWidth="1" min="54" max="54"/>
     <col width="21" customWidth="1" min="55" max="55"/>
     <col width="20" customWidth="1" min="56" max="56"/>
-    <col width="44" customWidth="1" min="57" max="57"/>
+    <col width="39" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1968,13 +1968,13 @@
         <v>14.27473646102501</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>5.154008617644307</v>
+        <v>5.154009202964633</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>2.016666460271793</v>
+        <v>2.016666231247005</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>0.1412752148369249</v>
+        <v>0.1412751987928607</v>
       </c>
       <c r="W2" s="2" t="n">
         <v>0.2</v>
@@ -2034,22 +2034,22 @@
         <v>0.05735188883641247</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>33.55516001704655</v>
+        <v>33.55515585102087</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>2.358833309808101</v>
+        <v>2.358833016948221</v>
       </c>
       <c r="AR2" s="3" t="n">
-        <v>3.802158477058641e+23</v>
+        <v>3.80215800500338e+23</v>
       </c>
       <c r="AS2" s="3" t="n">
-        <v>2.672810399443467e+22</v>
+        <v>2.672810067601905e+22</v>
       </c>
       <c r="AT2" s="3" t="n">
-        <v>2.421974949886355e+24</v>
+        <v>2.421974649187153e+24</v>
       </c>
       <c r="AU2" s="3" t="n">
-        <v>1.702721733277541e+23</v>
+        <v>1.702721521876897e+23</v>
       </c>
       <c r="AV2" s="2" t="n">
         <v>72.00105954340778</v>
@@ -2058,25 +2058,25 @@
         <v>5.061471842368986</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>2.145752233243117</v>
+        <v>2.145752499648045</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>0.8091065333821519</v>
+        <v>0.8091066252691731</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>0.1344870045787303</v>
+        <v>0.1344869893055761</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>33.27784805081173</v>
+        <v>33.2778476984484</v>
       </c>
       <c r="BB2" s="3" t="n">
-        <v>3.770736065641922e+23</v>
+        <v>3.770736025715389e+23</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>0.8333230135896473</v>
+        <v>0.8333115623502168</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>7.088298817298562</v>
+        <v>7.08829801230866</v>
       </c>
       <c r="BE2" t="inlineStr"/>
     </row>
@@ -2145,13 +2145,13 @@
         <v>1.343018729574148</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>0.9312119431632206</v>
+        <v>0.9312121114180388</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>1.494955678206653</v>
+        <v>1.49495540809258</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>1.113130923111312</v>
+        <v>1.113130721986736</v>
       </c>
       <c r="W3" s="2" t="n">
         <v>0.2</v>
@@ -2211,22 +2211,22 @@
         <v>0.08136520707143691</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>22.53191455512147</v>
+        <v>22.53191120265777</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>16.77758328145946</v>
+        <v>16.77758078516743</v>
       </c>
       <c r="AR3" s="3" t="n">
-        <v>2.553106880926642e+23</v>
+        <v>2.553106501056654e+23</v>
       </c>
       <c r="AS3" s="3" t="n">
-        <v>1.901079609387993e+23</v>
+        <v>1.90107932653141e+23</v>
       </c>
       <c r="AT3" s="3" t="n">
-        <v>1.626329083150271e+24</v>
+        <v>1.626328841173089e+24</v>
       </c>
       <c r="AU3" s="3" t="n">
-        <v>1.210988608292521e+24</v>
+        <v>1.210988428112744e+24</v>
       </c>
       <c r="AV3" s="2" t="n">
         <v>9.643540882980556</v>
@@ -2235,29 +2235,29 @@
         <v>7.180717372975728</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>0.4279947387244372</v>
+        <v>0.4279948024046465</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>0.1461871182359844</v>
+        <v>0.1461871446496136</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>0.7443495389517917</v>
+        <v>0.7443494044599881</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>30.14392317255951</v>
+        <v>30.14392413404001</v>
       </c>
       <c r="BB3" s="3" t="n">
-        <v>3.415628861973148e+23</v>
+        <v>3.415628970919171e+23</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-25.25221608966737</v>
+        <v>-25.25222959537099</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>55.65826049056668</v>
+        <v>55.65825043402813</v>
       </c>
       <c r="BE3" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -2326,13 +2326,13 @@
         <v>2.965581864565676</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>0.7726659251229667</v>
+        <v>0.7726660408861314</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>1.586994876839577</v>
+        <v>1.586994639071201</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>0.5351377737373639</v>
+        <v>0.5351376935614031</v>
       </c>
       <c r="W4" s="2" t="n">
         <v>0.2</v>
@@ -2392,22 +2392,22 @@
         <v>0.03246034689448935</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>22.69404816833188</v>
+        <v>22.69404562087823</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>7.653626631941197</v>
+        <v>7.653625772805842</v>
       </c>
       <c r="AR4" s="3" t="n">
-        <v>2.571478353200085e+23</v>
+        <v>2.571478064546343e+23</v>
       </c>
       <c r="AS4" s="3" t="n">
-        <v>8.672377471629875e+22</v>
+        <v>8.672376498137641e+22</v>
       </c>
       <c r="AT4" s="3" t="n">
-        <v>1.638031710988454e+24</v>
+        <v>1.638031527116021e+24</v>
       </c>
       <c r="AU4" s="3" t="n">
-        <v>5.524324399116141e+23</v>
+        <v>5.524323778999349e+23</v>
       </c>
       <c r="AV4" s="2" t="n">
         <v>8.494287505290718</v>
@@ -2416,29 +2416,29 @@
         <v>2.864720502381708</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>0.3742958260370648</v>
+        <v>0.3742958680525469</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>0.1212976334572946</v>
+        <v>0.1212976516304759</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>0.8970852188798589</v>
+        <v>0.8970850844758363</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>28.60002700642107</v>
+        <v>28.60002808095189</v>
       </c>
       <c r="BB4" s="3" t="n">
-        <v>3.240688915544655e+23</v>
+        <v>3.240689037300489e+23</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>-20.65025615802118</v>
+        <v>-20.65026804643995</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>26.76090700971318</v>
+        <v>26.7609030003131</v>
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -2507,13 +2507,13 @@
         <v>3.08952723080917</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>0.5046963530564196</v>
+        <v>0.5046963885603317</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>2.098043986084978</v>
+        <v>2.098043838493731</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>0.6790825357235919</v>
+        <v>0.6790824879521252</v>
       </c>
       <c r="W5" s="2" t="n">
         <v>0.2</v>
@@ -2573,22 +2573,22 @@
         <v>0.02690630628662187</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>27.48048356101584</v>
+        <v>27.48048213288326</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>8.896171048733246</v>
+        <v>8.896170586408347</v>
       </c>
       <c r="AR5" s="3" t="n">
-        <v>3.113832670507515e+23</v>
+        <v>3.11383250868482e+23</v>
       </c>
       <c r="AS5" s="3" t="n">
-        <v>1.00803131766087e+23</v>
+        <v>1.008031265274515e+23</v>
       </c>
       <c r="AT5" s="3" t="n">
-        <v>1.983511411113287e+24</v>
+        <v>1.983511308032231e+24</v>
       </c>
       <c r="AU5" s="3" t="n">
-        <v>6.421184660125047e+23</v>
+        <v>6.421184326422654e+23</v>
       </c>
       <c r="AV5" s="2" t="n">
         <v>7.33507277643852</v>
@@ -2597,25 +2597,25 @@
         <v>2.374560183019267</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>0.2669193487862835</v>
+        <v>0.2669193626578095</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>0.07923019671215378</v>
+        <v>0.07923020228576637</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>1.373394470481658</v>
+        <v>1.373394373867381</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>26.19628925158559</v>
+        <v>26.19628973302349</v>
       </c>
       <c r="BB5" s="3" t="n">
-        <v>2.968319721759537e+23</v>
+        <v>2.9683197763116e+23</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>4.902199304248881</v>
+        <v>4.902191924686525</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>33.95966109281979</v>
+        <v>33.95965870385714</v>
       </c>
       <c r="BE5" t="inlineStr"/>
     </row>
@@ -2684,13 +2684,13 @@
         <v>2.283321960425025</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>0.3649451288823548</v>
+        <v>0.3649451484627882</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>1.951217719221146</v>
+        <v>1.951217614532294</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>0.8545521626122056</v>
+        <v>0.8545521167628449</v>
       </c>
       <c r="W6" s="2" t="n">
         <v>0.2</v>
@@ -2750,22 +2750,22 @@
         <v>0.02448135121418641</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>24.85613971635959</v>
+        <v>24.85613882669739</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>10.88692400473625</v>
+        <v>10.88692361506654</v>
       </c>
       <c r="AR6" s="3" t="n">
-        <v>2.816466447529965e+23</v>
+        <v>2.816466346721723e+23</v>
       </c>
       <c r="AS6" s="3" t="n">
-        <v>1.233604917177341e+23</v>
+        <v>1.233604873023596e+23</v>
       </c>
       <c r="AT6" s="3" t="n">
-        <v>1.794089127076588e+24</v>
+        <v>1.794089062861738e+24</v>
       </c>
       <c r="AU6" s="3" t="n">
-        <v>7.858080146910282e+23</v>
+        <v>7.85807986565032e+23</v>
       </c>
       <c r="AV6" s="2" t="n">
         <v>4.93279394198141</v>
@@ -2774,29 +2774,29 @@
         <v>2.160550809184148</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>0.1984537421446335</v>
+        <v>0.1984537492477799</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>0.05729122902391755</v>
+        <v>0.05729123209776895</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>1.899318899481437</v>
+        <v>1.899318797577117</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>25.47756662058322</v>
+        <v>25.47756707562872</v>
       </c>
       <c r="BB6" s="3" t="n">
-        <v>2.886880761470529e+23</v>
+        <v>2.88688081303205e+23</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-2.439114038942717</v>
+        <v>-2.439119273385309</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>42.73141217474336</v>
+        <v>42.73140988207123</v>
       </c>
       <c r="BE6" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -2865,13 +2865,13 @@
         <v>4.506011387696815</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>0.3411182000345155</v>
+        <v>0.341118237048898</v>
       </c>
       <c r="U7" s="2" t="n">
-        <v>2.005247058533038</v>
+        <v>2.005246840945781</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>0.4450159766591252</v>
+        <v>0.4450159283709078</v>
       </c>
       <c r="W7" s="2" t="n">
         <v>0.2</v>
@@ -2931,22 +2931,22 @@
         <v>0.01191959782795906</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>25.48483186394954</v>
+        <v>25.48482990062792</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>5.657701413243935</v>
+        <v>5.657700977381238</v>
       </c>
       <c r="AR7" s="3" t="n">
-        <v>2.887703991240232e+23</v>
+        <v>2.887703768774895e+23</v>
       </c>
       <c r="AS7" s="3" t="n">
-        <v>6.410780749698084e+22</v>
+        <v>6.410780255819037e+22</v>
       </c>
       <c r="AT7" s="3" t="n">
-        <v>1.839467442420028e+24</v>
+        <v>1.839467300709608e+24</v>
       </c>
       <c r="AU7" s="3" t="n">
-        <v>4.08370137069058e+23</v>
+        <v>4.083701056087006e+23</v>
       </c>
       <c r="AV7" s="2" t="n">
         <v>4.738407978556136</v>
@@ -2955,25 +2955,25 @@
         <v>1.051939352000445</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>0.1859305175663731</v>
+        <v>0.1859305318902437</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>0.05355073783901342</v>
+        <v>0.05355074364974851</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>2.031985336724368</v>
+        <v>2.031985116235768</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>25.41814661241121</v>
+        <v>25.41814741232349</v>
       </c>
       <c r="BB7" s="3" t="n">
-        <v>2.880147839092471e+23</v>
+        <v>2.880147929731086e+23</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>0.2623529266518976</v>
+        <v>0.2623420472890149</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>22.25851278425384</v>
+        <v>22.25851036900594</v>
       </c>
       <c r="BE7" t="inlineStr"/>
     </row>
@@ -3042,13 +3042,13 @@
         <v>18.56896321259232</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>10.60366757376142</v>
+        <v>10.60366823249836</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>2.272062324113326</v>
+        <v>2.272062182964871</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>0.1223580604959438</v>
+        <v>0.1223580528946333</v>
       </c>
       <c r="W8" s="2" t="n">
         <v>0.2</v>
@@ -3108,22 +3108,22 @@
         <v>0.1039066067345771</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>54.51585733730867</v>
+        <v>54.51585293094176</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>2.953107821348059</v>
+        <v>2.953107582656471</v>
       </c>
       <c r="AR8" s="3" t="n">
-        <v>5.938387451996493e+23</v>
+        <v>5.938386972012958e+23</v>
       </c>
       <c r="AS8" s="3" t="n">
-        <v>3.216806868170546e+22</v>
+        <v>3.216806608164889e+22</v>
       </c>
       <c r="AT8" s="3" t="n">
-        <v>3.729307319853797e+24</v>
+        <v>3.729307018424138e+24</v>
       </c>
       <c r="AU8" s="3" t="n">
-        <v>2.020445630752459e+23</v>
+        <v>2.020445467445392e+23</v>
       </c>
       <c r="AV8" s="2" t="n">
         <v>176.0925657426108</v>
@@ -3132,25 +3132,25 @@
         <v>9.538882053311641</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>3.23011641645961</v>
+        <v>3.230116677541063</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>1.68848209773271</v>
+        <v>1.688482202627127</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>0.06536862606624197</v>
+        <v>0.06536862200531438</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>47.98799465906685</v>
+        <v>47.9879937615111</v>
       </c>
       <c r="BB8" s="3" t="n">
-        <v>5.227310350576718e+23</v>
+        <v>5.22731025280638e+23</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>13.60311620566632</v>
+        <v>13.60310914824357</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>6.153847107653829</v>
+        <v>6.153846725355332</v>
       </c>
       <c r="BE8" t="inlineStr"/>
     </row>
@@ -3219,13 +3219,13 @@
         <v>2.486864471799392</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>1.077177410724217</v>
+        <v>1.077177645548336</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>2.750780878065064</v>
+        <v>2.750780278396386</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>1.106124161271528</v>
+        <v>1.106123920137085</v>
       </c>
       <c r="W9" s="2" t="n">
         <v>0.2</v>
@@ -3285,22 +3285,22 @@
         <v>0.09487403505582533</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>46.63926857927817</v>
+        <v>46.63926122130088</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>18.75622820675455</v>
+        <v>18.75622524770512</v>
       </c>
       <c r="AR9" s="3" t="n">
-        <v>5.080394234430154e+23</v>
+        <v>5.080393432929047e+23</v>
       </c>
       <c r="AS9" s="3" t="n">
-        <v>2.043107375907456e+23</v>
+        <v>2.043107053579552e+23</v>
       </c>
       <c r="AT9" s="3" t="n">
-        <v>3.190487579222137e+24</v>
+        <v>3.190487075879441e+24</v>
       </c>
       <c r="AU9" s="3" t="n">
-        <v>1.283074784750438e+24</v>
+        <v>1.283074582327986e+24</v>
       </c>
       <c r="AV9" s="2" t="n">
         <v>21.65747945676702</v>
@@ -3309,29 +3309,29 @@
         <v>8.709669757872257</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>0.4643614729925126</v>
+        <v>0.4643615462518457</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>0.1715250654019454</v>
+        <v>0.171525102794321</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>0.6434846977471635</v>
+        <v>0.6434845574678629</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>33.90983916689493</v>
+        <v>33.90984120948404</v>
       </c>
       <c r="BB9" s="3" t="n">
-        <v>3.693783299819775e+23</v>
+        <v>3.693783522318075e+23</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>37.53904390325319</v>
+        <v>37.53901391981928</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>55.31205298391873</v>
+        <v>55.31204092592242</v>
       </c>
       <c r="BE9" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -3400,13 +3400,13 @@
         <v>4.72630225289397</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>0.8527863757903911</v>
+        <v>0.8527865423494825</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>2.226666134189018</v>
+        <v>2.226665699295326</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>0.4711222463238791</v>
+        <v>0.4711221543082463</v>
       </c>
       <c r="W10" s="2" t="n">
         <v>0.2</v>
@@ -3466,22 +3466,22 @@
         <v>0.03199999790477622</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>35.02344379374568</v>
+        <v>35.02343934375751</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>7.413154973750841</v>
+        <v>7.413154031854545</v>
       </c>
       <c r="AR10" s="3" t="n">
-        <v>3.81508774343622e+23</v>
+        <v>3.81508725870104e+23</v>
       </c>
       <c r="AS10" s="3" t="n">
-        <v>8.075115870130545e+22</v>
+        <v>8.07511484412721e+22</v>
       </c>
       <c r="AT10" s="3" t="n">
-        <v>2.395875102877946e+24</v>
+        <v>2.395874798464253e+24</v>
       </c>
       <c r="AU10" s="3" t="n">
-        <v>5.071220601615798e+23</v>
+        <v>5.071219957279627e+23</v>
       </c>
       <c r="AV10" s="2" t="n">
         <v>13.87905939732096</v>
@@ -3490,25 +3490,25 @@
         <v>2.937678510661091</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>0.396279117469294</v>
+        <v>0.3962791678195</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>0.1357940088838202</v>
+        <v>0.1357940354059685</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>0.8128028310929724</v>
+        <v>0.8128026723431629</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>31.45819057108147</v>
+        <v>31.45819271823463</v>
       </c>
       <c r="BB10" s="3" t="n">
-        <v>3.426726337512406e+23</v>
+        <v>3.42672657140082e+23</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>11.33330670945089</v>
+        <v>11.33328496476627</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>23.56510288473338</v>
+        <v>23.56509828219578</v>
       </c>
       <c r="BE10" t="inlineStr"/>
     </row>
@@ -3577,13 +3577,13 @@
         <v>2.426398437512705</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>0.5108042920535788</v>
+        <v>0.5108043375662259</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>1.814095898955189</v>
+        <v>1.814095737319313</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>0.7476496320261458</v>
+        <v>0.7476495654105919</v>
       </c>
       <c r="W11" s="2" t="n">
         <v>0.2</v>
@@ -3643,22 +3643,22 @@
         <v>0.03040932029135026</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>24.89584820661005</v>
+        <v>24.89584672782507</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>10.26144449507104</v>
+        <v>10.26144388555294</v>
       </c>
       <c r="AR11" s="3" t="n">
-        <v>2.71189337961242e+23</v>
+        <v>2.711893218529047e+23</v>
       </c>
       <c r="AS11" s="3" t="n">
-        <v>1.117774464260065e+23</v>
+        <v>1.117774397865537e+23</v>
       </c>
       <c r="AT11" s="3" t="n">
-        <v>1.7030690423966e+24</v>
+        <v>1.703068941236241e+24</v>
       </c>
       <c r="AU11" s="3" t="n">
-        <v>7.01964109697502e+23</v>
+        <v>7.019640680016345e+23</v>
       </c>
       <c r="AV11" s="2" t="n">
         <v>6.772974748003384</v>
@@ -3667,29 +3667,29 @@
         <v>2.791650393526319</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>0.2720523796495957</v>
+        <v>0.2720523958091977</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>0.08133826306585649</v>
+        <v>0.08133827031309329</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>1.35697211504096</v>
+        <v>1.356971994134796</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>27.44711370655606</v>
+        <v>27.44711452176567</v>
       </c>
       <c r="BB11" s="3" t="n">
-        <v>2.989801565809512e+23</v>
+        <v>2.989801654609924e+23</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>-9.295205052240533</v>
+        <v>-9.295213134034318</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>37.38624251999208</v>
+        <v>37.38623918887929</v>
       </c>
       <c r="BE11" t="inlineStr">
         <is>
-          <t>LAC &lt; 3 sigma: HVL/TVL/MFP guvenilir degil</t>
+          <t>LAC &lt; 3σ: HVL/TVL/MFP güvenilir değil</t>
         </is>
       </c>
     </row>
@@ -3758,13 +3758,13 @@
         <v>4.014687427582307</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>0.3586335710374853</v>
+        <v>0.3586335981033563</v>
       </c>
       <c r="U12" s="2" t="n">
-        <v>1.98440994091548</v>
+        <v>1.984409791153206</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>0.4942875321455638</v>
+        <v>0.4942874948419686</v>
       </c>
       <c r="W12" s="2" t="n">
         <v>0.2</v>
@@ -3824,22 +3824,22 @@
         <v>0.0141175893920553</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>26.0057754835553</v>
+        <v>26.00577438549107</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>6.479442794883083</v>
+        <v>6.479442521295995</v>
       </c>
       <c r="AR12" s="3" t="n">
-        <v>2.832797251182455e+23</v>
+        <v>2.83279713157082e+23</v>
       </c>
       <c r="AS12" s="3" t="n">
-        <v>7.058027456303109e+22</v>
+        <v>7.058027158285944e+22</v>
       </c>
       <c r="AT12" s="3" t="n">
-        <v>1.778996673742582e+24</v>
+        <v>1.778996598626475e+24</v>
       </c>
       <c r="AU12" s="3" t="n">
-        <v>4.432471416723907e+23</v>
+        <v>4.432471229567854e+23</v>
       </c>
       <c r="AV12" s="2" t="n">
         <v>5.201720485954501</v>
@@ -3848,25 +3848,25 @@
         <v>1.296029427964047</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>0.2000217409107372</v>
+        <v>0.2000217493564276</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>0.05710725653463142</v>
+        <v>0.05710726084448348</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>1.932744830760687</v>
+        <v>1.932744684897548</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>26.21008386156128</v>
+        <v>26.21008473293036</v>
       </c>
       <c r="BB12" s="3" t="n">
-        <v>2.855052469527121e+23</v>
+        <v>2.855052564444956e+23</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>-0.7795029542259957</v>
+        <v>-0.7795104423397278</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>24.72118299623447</v>
+        <v>24.72118113054103</v>
       </c>
       <c r="BE12" t="inlineStr"/>
     </row>
@@ -3935,13 +3935,13 @@
         <v>5.419111152478443</v>
       </c>
       <c r="T13" s="2" t="n">
-        <v>0.3343770710786853</v>
+        <v>0.3343771199217104</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>2.099834227483437</v>
+        <v>2.099833920757139</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>0.3874868347225305</v>
+        <v>0.3874867781216805</v>
       </c>
       <c r="W13" s="2" t="n">
         <v>0.2</v>
@@ -4001,22 +4001,22 @@
         <v>0.01032099685219263</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>27.41445242844401</v>
+        <v>27.41444997949892</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>5.061384852047949</v>
+        <v>5.061384399912215</v>
       </c>
       <c r="AR13" s="3" t="n">
-        <v>2.9862437876954e+23</v>
+        <v>2.986243520932929e+23</v>
       </c>
       <c r="AS13" s="3" t="n">
-        <v>5.51334341293705e+22</v>
+        <v>5.513342920427659e+22</v>
       </c>
       <c r="AT13" s="3" t="n">
-        <v>1.875361098672711e+24</v>
+        <v>1.87536093114588e+24</v>
       </c>
       <c r="AU13" s="3" t="n">
-        <v>3.462422589469427e+23</v>
+        <v>3.462422280169695e+23</v>
       </c>
       <c r="AV13" s="2" t="n">
         <v>5.131994436526965</v>
@@ -4025,25 +4025,25 @@
         <v>0.947492895203022</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>0.1872003261754824</v>
+        <v>0.1872003428981714</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>0.05324475654119191</v>
+        <v>0.0532447643187437</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>2.072950691038366</v>
+        <v>2.072950388238991</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>26.11106350171183</v>
+        <v>26.11106498328598</v>
       </c>
       <c r="BB13" s="3" t="n">
-        <v>2.844266226933817e+23</v>
+        <v>2.844266388321013e+23</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>4.991711374171827</v>
+        <v>4.991696037856935</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>19.38406243666072</v>
+        <v>19.38405960519829</v>
       </c>
       <c r="BE13" t="inlineStr"/>
     </row>
@@ -6622,14 +6622,14 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
@@ -6716,34 +6716,34 @@
         <v>80.89906428571429</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.8091065333821519</v>
+        <v>0.8091066252691731</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>71.40601677255438</v>
+        <v>71.40602488185262</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2.145752233243117</v>
+        <v>2.145752499648045</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>33.27784805081173</v>
+        <v>33.2778476984484</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>3.770736065641922e+23</v>
+        <v>3.770736025715389e+23</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>5.154008617644307</v>
+        <v>5.154009202964633</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.1344870045787303</v>
+        <v>0.1344869893055761</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0.4467561589073295</v>
+        <v>0.4467561081710095</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0.1940237345697455</v>
+        <v>0.1940237125352417</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>2.401958873813904e+24</v>
+        <v>2.401958848380703e+24</v>
       </c>
     </row>
     <row r="3">
@@ -6761,34 +6761,34 @@
         <v>295.4176231113203</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.1461871182359844</v>
+        <v>0.1461871446496136</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12.90144052236912</v>
+        <v>12.90144285344911</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.4279947387244372</v>
+        <v>0.4279948024046465</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>30.14392317255951</v>
+        <v>30.14392413404001</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3.415628861973148e+23</v>
+        <v>3.415628970919171e+23</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.9312119431632206</v>
+        <v>0.9312121114180388</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.7443495389517917</v>
+        <v>0.7443494044599881</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2.472675645860412</v>
+        <v>2.472675199088311</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>1.073869388533736</v>
+        <v>1.073869194503078</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>2.175755585076895e+24</v>
+        <v>2.175755654475512e+24</v>
       </c>
     </row>
     <row r="4">
@@ -6806,34 +6806,34 @@
         <v>359.5183270178899</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.1212976334572946</v>
+        <v>0.1212976516304759</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10.70487073305073</v>
+        <v>10.7048723368871</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.3742958260370648</v>
+        <v>0.3742958680525469</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>28.60002700642107</v>
+        <v>28.60002808095189</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3.240688915544655e+23</v>
+        <v>3.240689037300489e+23</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.7726659251229667</v>
+        <v>0.7726660408861314</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.8970852188798589</v>
+        <v>0.8970850844758363</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>2.980052592105182</v>
+        <v>2.980052145624684</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1.294220396532763</v>
+        <v>1.294220202628746</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>2.064318839201945e+24</v>
+        <v>2.064318916760411e+24</v>
       </c>
     </row>
     <row r="5">
@@ -6851,34 +6851,34 @@
         <v>661.657</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.07923019671215378</v>
+        <v>0.07923020228576637</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>6.992296467650345</v>
+        <v>6.992296959537949</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.2669193487862835</v>
+        <v>0.2669193626578095</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>26.19628925158559</v>
+        <v>26.19628973302349</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>2.968319721759537e+23</v>
+        <v>2.9683197763116e+23</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.5046963530564196</v>
+        <v>0.5046963885603317</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.373394470481658</v>
+        <v>1.373394373867381</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>4.562317676855972</v>
+        <v>4.562317355910292</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>1.981389391748212</v>
+        <v>1.981389252363274</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>1.890819662760825e+24</v>
+        <v>1.890819697510489e+24</v>
       </c>
     </row>
     <row r="6">
@@ -6896,34 +6896,34 @@
         <v>1173.228</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.05729122902391755</v>
+        <v>0.05729123209776895</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.056118436593945</v>
+        <v>5.056118707870315</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.1984537421446335</v>
+        <v>0.1984537492477799</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25.47756662058322</v>
+        <v>25.47756707562872</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>2.886880761470529e+23</v>
+        <v>2.88688081303205e+23</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.3649451288823548</v>
+        <v>0.3649451484627882</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1.899318899481437</v>
+        <v>1.899318797577117</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>6.309400813337932</v>
+        <v>6.309400474819109</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>2.740137957348553</v>
+        <v>2.740137810331696</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1.838943045056727e+24</v>
+        <v>1.838943077901416e+24</v>
       </c>
     </row>
     <row r="7">
@@ -6941,34 +6941,34 @@
         <v>1332.492</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.05355073783901342</v>
+        <v>0.05355074364974851</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.72600915522357</v>
+        <v>4.726009668037928</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.1859305175663731</v>
+        <v>0.1859305318902437</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25.41814661241121</v>
+        <v>25.41814741232349</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>2.880147839092471e+23</v>
+        <v>2.880147929731086e+23</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.3411182000345155</v>
+        <v>0.341118237048898</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>2.031985336724368</v>
+        <v>2.031985116235768</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>6.750109178463837</v>
+        <v>6.750108446016561</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>2.931535168451336</v>
+        <v>2.931534850353527</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>1.834654173501904e+24</v>
+        <v>1.834654231238702e+24</v>
       </c>
     </row>
     <row r="8">
@@ -6986,34 +6986,34 @@
         <v>80.89906428571429</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1.68848209773271</v>
+        <v>1.688482202627127</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>155.0068093412279</v>
+        <v>155.0068189707935</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>3.23011641645961</v>
+        <v>3.230116677541063</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>47.98799465906685</v>
+        <v>47.9879937615111</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>5.227310350576718e+23</v>
+        <v>5.22731025280638e+23</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>10.60366757376142</v>
+        <v>10.60366823249836</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.06536862606624197</v>
+        <v>0.06536862200531438</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0.2171498754536356</v>
+        <v>0.2171498619635261</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0.09430699265549232</v>
+        <v>0.09430698679681221</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3.282750900162179e+24</v>
+        <v>3.282750838762406e+24</v>
       </c>
     </row>
     <row r="9">
@@ -7031,34 +7031,34 @@
         <v>295.4176231113203</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.1715250654019454</v>
+        <v>0.171525102794321</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>15.74642286447853</v>
+        <v>15.74642629719057</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.4643614729925126</v>
+        <v>0.4643615462518457</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>33.90983916689493</v>
+        <v>33.90984120948404</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.693783299819775e+23</v>
+        <v>3.693783522318075e+23</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.077177410724217</v>
+        <v>1.077177645548336</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.6434846977471635</v>
+        <v>0.6434845574678629</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>2.137609896076405</v>
+        <v>2.137609430078656</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0.9283521823277665</v>
+        <v>0.9283519799475151</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>2.319695912286819e+24</v>
+        <v>2.319696052015751e+24</v>
       </c>
     </row>
     <row r="10">
@@ -7076,34 +7076,34 @@
         <v>359.5183270178899</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.1357940088838202</v>
+        <v>0.1357940354059685</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>12.46622399668903</v>
+        <v>12.46622643148747</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.396279117469294</v>
+        <v>0.3962791678195</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>31.45819057108147</v>
+        <v>31.45819271823463</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>3.426726337512406e+23</v>
+        <v>3.42672657140082e+23</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.8527863757903911</v>
+        <v>0.8527865423494825</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.8128028310929724</v>
+        <v>0.8128026723431629</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>2.700072560211733</v>
+        <v>2.700072032856281</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>1.172626613638341</v>
+        <v>1.172626384610778</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>2.151984139957791e+24</v>
+        <v>2.151984286839715e+24</v>
       </c>
     </row>
     <row r="11">
@@ -7121,34 +7121,34 @@
         <v>661.657</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.08133826306585649</v>
+        <v>0.08133827031309329</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>7.467052598381609</v>
+        <v>7.467053263695772</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.2720523796495957</v>
+        <v>0.2720523958091977</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27.44711370655606</v>
+        <v>27.44711452176567</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>2.989801565809512e+23</v>
+        <v>2.989801654609924e+23</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.5108042920535788</v>
+        <v>0.5108043375662259</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1.35697211504096</v>
+        <v>1.356971994134796</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>4.507763792933293</v>
+        <v>4.50776339129171</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>1.957696940994202</v>
+        <v>1.957696766563479</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>1.877595383328374e+24</v>
+        <v>1.877595439095032e+24</v>
       </c>
     </row>
     <row r="12">
@@ -7166,34 +7166,34 @@
         <v>1173.228</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.05710725653463142</v>
+        <v>0.05710726084448348</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5.242586603405906</v>
+        <v>5.242586999060926</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.2000217409107372</v>
+        <v>0.2000217493564276</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>26.21008386156128</v>
+        <v>26.21008473293036</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>2.855052469527121e+23</v>
+        <v>2.855052564444956e+23</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.3586335710374853</v>
+        <v>0.3586335981033563</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1.932744830760687</v>
+        <v>1.932744684897548</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>6.420439353552246</v>
+        <v>6.420438869005389</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>2.788361382642222</v>
+        <v>2.788361172206195</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>1.792972950863032e+24</v>
+        <v>1.792973010471432e+24</v>
       </c>
     </row>
     <row r="13">
@@ -7211,34 +7211,34 @@
         <v>1332.492</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.05324475654119191</v>
+        <v>0.0532447643187437</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>4.887999604309189</v>
+        <v>4.888000318307571</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.1872003261754824</v>
+        <v>0.1872003428981714</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>26.11106350171183</v>
+        <v>26.11106498328598</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>2.844266226933817e+23</v>
+        <v>2.844266388321013e+23</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.3343770710786853</v>
+        <v>0.3343771199217104</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2.072950691038366</v>
+        <v>2.072950388238991</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>6.88619313987652</v>
+        <v>6.886192133998771</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>2.9906356819684</v>
+        <v>2.990635245121244</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>1.786199190514437e+24</v>
+        <v>1.786199291865596e+24</v>
       </c>
     </row>
   </sheetData>
@@ -7319,13 +7319,13 @@
         <v>80.89906428571429</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.352557616883219</v>
+        <v>2.35255765896867</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>26.70152895162454</v>
+        <v>26.70152942929441</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.02595908203667767</v>
+        <v>0.02595908157228962</v>
       </c>
     </row>
     <row r="3">
@@ -7346,13 +7346,13 @@
         <v>295.4176231113203</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.4163622880996919</v>
+        <v>0.4163623946355609</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>4.725711969931503</v>
+        <v>4.725713179113615</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.1466757146796639</v>
+        <v>0.1466756771493179</v>
       </c>
     </row>
     <row r="4">
@@ -7373,13 +7373,13 @@
         <v>359.5183270178899</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.2821304751238382</v>
+        <v>0.2821305555687182</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3.202180892655563</v>
+        <v>3.202181805704951</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.2164609695066663</v>
+        <v>0.2164609077863869</v>
       </c>
     </row>
     <row r="5">
@@ -7400,13 +7400,13 @@
         <v>661.657</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.1102033533310854</v>
+        <v>0.1102033739037272</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1.250808060307819</v>
+        <v>1.250808293807304</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.554159509005214</v>
+        <v>0.5541594055553406</v>
       </c>
     </row>
     <row r="6">
@@ -7427,13 +7427,13 @@
         <v>1173.228</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.06166367792142712</v>
+        <v>0.06166369276333716</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.6998827444081978</v>
+        <v>0.6998829128638767</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.9903761538599614</v>
+        <v>0.9903759154851071</v>
       </c>
     </row>
     <row r="7">
@@ -7454,13 +7454,13 @@
         <v>1332.492</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.05610115372288973</v>
+        <v>0.05610117871916188</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.6367480947547984</v>
+        <v>0.6367483784624873</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1.088573623179611</v>
+        <v>1.088573138158028</v>
       </c>
     </row>
     <row r="8">
@@ -7481,13 +7481,13 @@
         <v>80.89906428571429</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.1996495265144275</v>
+        <v>0.1996495455767022</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.4591939109831832</v>
+        <v>0.459193954826415</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>1.509486872497597</v>
+        <v>1.509486728373786</v>
       </c>
     </row>
     <row r="9">
@@ -7508,13 +7508,13 @@
         <v>295.4176231113203</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.1103931810472376</v>
+        <v>0.1103931815987268</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.2539043164086464</v>
+        <v>0.2539043176770715</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2.729954300754617</v>
+        <v>2.729954287116635</v>
       </c>
     </row>
     <row r="10">
@@ -7535,13 +7535,13 @@
         <v>359.5183270178899</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.1020581609644876</v>
+        <v>0.1020581627180894</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.2347337702183215</v>
+        <v>0.2347337742516055</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2.952907798120663</v>
+        <v>2.952907747382689</v>
       </c>
     </row>
     <row r="11">
@@ -7562,13 +7562,13 @@
         <v>661.657</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.07883704400614537</v>
+        <v>0.07883704636894012</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.1813252012141343</v>
+        <v>0.1813252066485623</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>3.822674266559227</v>
+        <v>3.822674151991329</v>
       </c>
     </row>
     <row r="12">
@@ -7589,13 +7589,13 @@
         <v>1173.228</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.05993790771013759</v>
+        <v>0.059937908254028</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.1378571877333165</v>
+        <v>0.1378571889842644</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>5.028008999435216</v>
+        <v>5.028008953809903</v>
       </c>
     </row>
     <row r="13">
@@ -7616,13 +7616,13 @@
         <v>1332.492</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.05619604576989413</v>
+        <v>0.05619604768884361</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.1292509052707565</v>
+        <v>0.1292509096843403</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>5.36280329416596</v>
+        <v>5.362803111040117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>